<commit_message>
Update schematic assignment and add in RC servos
</commit_message>
<xml_diff>
--- a/docs/Appendix/03-Power-Budget/DirksPowerBudget.xlsx
+++ b/docs/Appendix/03-Power-Budget/DirksPowerBudget.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Precision\Desktop\J2DIndivGithub\Classwork\JacobDirksEGR314.github.io\docs\Appendix\03-Power-Budget\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{857DAD5D-2939-4EF6-AFB0-F69557C7C322}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{761BFCDD-2F88-418A-B02B-E96F1C314B8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14400" yWindow="0" windowWidth="14400" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Power Budget" sheetId="1" r:id="rId1"/>
@@ -1431,11 +1431,11 @@
         <v>1</v>
       </c>
       <c r="F27" s="27">
-        <v>1000</v>
+        <v>6000</v>
       </c>
       <c r="G27" s="28">
         <f>E27*F27</f>
-        <v>1000</v>
+        <v>6000</v>
       </c>
       <c r="H27" s="16" t="s">
         <v>14</v>
@@ -1452,7 +1452,7 @@
       <c r="F28" s="47"/>
       <c r="G28" s="28">
         <f>G27-G25</f>
-        <v>-562.5</v>
+        <v>4437.5</v>
       </c>
       <c r="H28" s="16" t="s">
         <v>14</v>

</xml_diff>